<commit_message>
Expand all features with comprehensive test cases: integration, regression, security, edge cases, boundary values, equivalence partitioning — 776 total test cases
</commit_message>
<xml_diff>
--- a/Advanced_Search/Advanced_Search_Test_Cases.xlsx
+++ b/Advanced_Search/Advanced_Search_Test_Cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1757,6 +1757,725 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AS_036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Integration: Advanced Search with Message List</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Verify search result navigates to correct message in conversation</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a keyword.
+2. Tap on a result.
+3. Verify the message in context.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Should navigate to the exact conversation and scroll to the matching message. Message should be highlighted.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>AS_037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Integration: Advanced Search with Conversation List</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Verify search results reflect recently sent messages</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>1. Send a new message with unique keyword.
+2. Immediately search for that keyword.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Newly sent message should appear in search results.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>AS_038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Regression: Advanced Search</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Verify search results after deleting a message</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a keyword.
+2. Delete a message containing that keyword.
+3. Search again.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Deleted message should no longer appear in search results.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>AS_039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Verify search results after editing a message</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for 'hello'.
+2. Edit a message from 'hello' to 'goodbye'.
+3. Search 'hello' again.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>'hello' result should disappear. Searching 'goodbye' should show the edited message.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>AS_040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Verify search works after app restart</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>1. Close and reopen app.
+2. Perform advanced search.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Search should work correctly with all historical data accessible.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>AS_041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Security: Advanced Search</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Verify search does not return messages from other users' private conversations</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a common keyword.
+2. Observe results.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Results should only include messages from conversations the user is a participant of.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AS_042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Verify XSS prevention in search input</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>1. Type '&lt;script&gt;alert(1)&lt;/script&gt;' in search field.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Script should not execute. Input should be sanitized.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>AS_043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Verify search input sanitization against injection</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1. Type SQL/NoSQL injection payloads in search field.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Search should handle gracefully. No server errors or data exposure.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>AS_044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Edge Case: Advanced Search</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with single character</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for 'a'.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Should return results or show minimum character requirement message.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>AS_045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with 500+ character query</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>1. Paste a very long string (500+ chars) in search.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Search should handle gracefully — truncate input or show max length warning.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Low / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>AS_046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with only emojis</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for '😀🎉'.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Should return messages containing those emojis or show no results.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Low / Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>AS_047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with unicode/multilingual text</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for text in Chinese/Arabic/Hindi/Japanese.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Should return matching messages in those languages correctly.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>AS_048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Verify search during high server load</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>1. Perform search during peak usage.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Search should complete (may be slower) or show timeout message. No crash.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>AS_049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Verify rapid consecutive searches</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>1. Type and search rapidly, changing keywords every second.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>App should debounce requests. Only latest search results should display. No race conditions.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>AS_050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Boundary: Advanced Search</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Verify search returning exactly 0 results</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a unique string that doesn't exist.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Empty state should display with 'No results found' message.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>AS_051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Verify search returning exactly 1 result</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a unique keyword that exists in only one message.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Single result should display correctly with all details.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>AS_052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Verify search returning 1000+ results</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a very common word like 'the' or 'hi'.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Results should load with pagination/infinite scroll. Performance should be acceptable.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>AS_053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Equivalence Partitioning: Search Query Types</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with alphabetic characters only</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for 'hello'.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Should return matching text messages.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>AS_054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with numeric characters only</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for '12345'.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Should return messages containing that number.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>AS_055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with alphanumeric mix</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for 'test123'.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Should return messages containing 'test123'.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>AS_056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with special characters</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for '@#$%'.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Should handle gracefully — return matching results or empty state.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Low / Medium</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split all test case files into separate sheets per testing type: Functional, Integration, Regression, Security, Edge Cases, Boundary Values, Equivalence Partitioning
</commit_message>
<xml_diff>
--- a/Advanced_Search/Advanced_Search_Test_Cases.xlsx
+++ b/Advanced_Search/Advanced_Search_Test_Cases.xlsx
@@ -7,7 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Advanced Search Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Functional" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Integration" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regression" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Security" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Edge Cases" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Boundary Values" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Equivalence Partitioning" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,10 +439,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="004472C4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -540,9 +547,9 @@
           <t>AS_002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify advanced search panel opens</t>
@@ -570,9 +577,9 @@
           <t>AS_003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search input field in advanced search</t>
@@ -601,9 +608,9 @@
           <t>AS_004</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Verify closing advanced search panel</t>
@@ -675,9 +682,9 @@
           <t>AS_006</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Verify audio result shows sender and conversation info</t>
@@ -706,9 +713,9 @@
           <t>AS_007</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Verify tapping audio result opens conversation</t>
@@ -823,9 +830,9 @@
           <t>AS_010</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Verify document result shows file details</t>
@@ -854,9 +861,9 @@
           <t>AS_011</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Verify tapping document result opens conversation</t>
@@ -971,9 +978,9 @@
           <t>AS_014</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr"/>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Verify photo thumbnails display correctly</t>
@@ -1002,9 +1009,9 @@
           <t>AS_015</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr"/>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Verify tapping photo result opens conversation</t>
@@ -1033,9 +1040,9 @@
           <t>AS_016</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr"/>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Verify photo preview from search results</t>
@@ -1150,9 +1157,9 @@
           <t>AS_019</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Verify video result shows thumbnail and duration</t>
@@ -1181,9 +1188,9 @@
           <t>AS_020</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr"/>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Verify tapping video result opens conversation</t>
@@ -1298,9 +1305,9 @@
           <t>AS_023</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Verify link result shows URL and preview</t>
@@ -1329,9 +1336,9 @@
           <t>AS_024</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr"/>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Verify tapping link result opens conversation</t>
@@ -1447,9 +1454,9 @@
           <t>AS_027</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Verify text search is case-insensitive</t>
@@ -1478,9 +1485,9 @@
           <t>AS_028</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Verify text search highlights matching text</t>
@@ -1509,9 +1516,9 @@
           <t>AS_029</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Verify partial text search</t>
@@ -1539,9 +1546,9 @@
           <t>AS_030</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr"/>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Verify tapping text result opens conversation</t>
@@ -1613,9 +1620,9 @@
           <t>AS_032</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Verify search with special characters</t>
@@ -1688,9 +1695,9 @@
           <t>AS_034</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr"/>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
       <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Verify search results pagination/infinite scroll</t>
@@ -1757,720 +1764,1122 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0070AD47"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_036</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Integration: Advanced Search with Message List</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search result navigates to correct message in conversation</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for a keyword.
 2. Tap on a result.
 3. Verify the message in context.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Should navigate to the exact conversation and scroll to the matching message. Message should be highlighted.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_037</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Integration: Advanced Search with Conversation List</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify search results reflect recently sent messages</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Send a new message with unique keyword.
 2. Immediately search for that keyword.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Newly sent message should appear in search results.</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FFC000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_038</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Regression: Advanced Search</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search results after deleting a message</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for a keyword.
 2. Delete a message containing that keyword.
 3. Search again.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Deleted message should no longer appear in search results.</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_039</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify search results after editing a message</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Search for 'hello'.
 2. Edit a message from 'hello' to 'goodbye'.
 3. Search 'hello' again.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>'hello' result should disappear. Searching 'goodbye' should show the edited message.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AS_040</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search works after app restart</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Close and reopen app.
 2. Perform advanced search.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Search should work correctly with all historical data accessible.</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF0000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_041</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Security: Advanced Search</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search does not return messages from other users' private conversations</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for a common keyword.
 2. Observe results.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Results should only include messages from conversations the user is a participant of.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>High / Critical</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_042</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr"/>
-      <c r="C43" s="2" t="inlineStr"/>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify XSS prevention in search input</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Type '&lt;script&gt;alert(1)&lt;/script&gt;' in search field.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Script should not execute. Input should be sanitized.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>High / Critical</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AS_043</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search input sanitization against injection</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Type SQL/NoSQL injection payloads in search field.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Search should handle gracefully. No server errors or data exposure.</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>High / Critical</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00ED7D31"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_044</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Edge Case: Advanced Search</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search with single character</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for 'a'.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Should return results or show minimum character requirement message.</t>
         </is>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_045</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify search with 500+ character query</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Paste a very long string (500+ chars) in search.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Search should handle gracefully — truncate input or show max length warning.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Low / Medium</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AS_046</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr"/>
-      <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search with only emojis</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Search for '😀🎉'.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Should return messages containing those emojis or show no results.</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Low / Low</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>AS_047</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Verify search with unicode/multilingual text</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>1. Search for text in Chinese/Arabic/Hindi/Japanese.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Should return matching messages in those languages correctly.</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>AS_048</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr"/>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Verify search during high server load</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>1. Perform search during peak usage.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Search should complete (may be slower) or show timeout message. No crash.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Medium / High</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>AS_049</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Verify rapid consecutive searches</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>1. Type and search rapidly, changing keywords every second.</t>
         </is>
       </c>
-      <c r="G50" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>App should debounce requests. Only latest search results should display. No race conditions.</t>
         </is>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Medium / High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_050</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Boundary: Advanced Search</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search returning exactly 0 results</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for a unique string that doesn't exist.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Empty state should display with 'No results found' message.</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_051</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify search returning exactly 1 result</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Search for a unique keyword that exists in only one message.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Single result should display correctly with all details.</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AS_052</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr"/>
-      <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search returning 1000+ results</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Search for a very common word like 'the' or 'hi'.</t>
         </is>
       </c>
-      <c r="G53" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Results should load with pagination/infinite scroll. Performance should be acceptable.</t>
         </is>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0000B0F0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>AS_053</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Equivalence Partitioning: Search Query Types</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Verify search with alphabetic characters only</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>1. Search for 'hello'.</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Should return matching text messages.</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>AS_054</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr"/>
-      <c r="C55" s="2" t="inlineStr"/>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Verify search with numeric characters only</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Search for '12345'.</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Should return messages containing that number.</t>
         </is>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>AS_055</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Verify search with alphanumeric mix</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>1. Search for 'test123'.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Should return messages containing 'test123'.</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>AS_056</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr"/>
-      <c r="C57" s="2" t="inlineStr"/>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Verify search with special characters</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>1. Search for '@#$%'.</t>
         </is>
       </c>
-      <c r="G57" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Should handle gracefully — return matching results or empty state.</t>
         </is>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Low / Medium</t>
         </is>

</xml_diff>

<commit_message>
Add blank row separators between Positive and Negative test cases in all sheets for clear visual separation
</commit_message>
<xml_diff>
--- a/Advanced_Search/Advanced_Search_Test_Cases.xlsx
+++ b/Advanced_Search/Advanced_Search_Test_Cases.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -739,341 +739,245 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>AS_008</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Verify Audio Search</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>User is logged in with no audio messages</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Verify empty state for audio search</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
 2. Select 'Audio' filter.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empty state message should display (e.g., 'No audio messages found').</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>AS_009</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Verify Documents Search</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has document messages in conversations</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Verify documents filter displays document messages</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Documents' filter.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>All document/file messages across conversations should display in results.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>AS_010</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="n"/>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AS_009</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Verify Documents Search</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has document messages in conversations</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Verify documents filter displays document messages</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Documents' filter.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>All document/file messages across conversations should display in results.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>AS_010</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Verify document result shows file details</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>1. Select 'Documents' filter.
 2. Observe results.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Each result should show file name, file type icon, size, sender, and date.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>AS_011</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Verify tapping document result opens conversation</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>1. Select 'Documents' filter.
 2. Tap on a document result.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Should navigate to the conversation and highlight/scroll to the document message.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>AS_012</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Verify Documents Search</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no document messages</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty state for documents search</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Documents' filter.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Empty state message should display (e.g., 'No documents found').</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>AS_013</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Verify Photos Search</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has image messages in conversations</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Verify photos filter displays image messages</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Photos' filter.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>All image messages across conversations should display as a grid/list.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>AS_014</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="n"/>
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Verify photo thumbnails display correctly</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Photos' filter.
-2. Observe results.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Photo thumbnails should load and display correctly with sender and date info.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>AS_015</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
+          <t>AS_012</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Verify Documents Search</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no document messages</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping photo result opens conversation</t>
+          <t>Verify empty state for documents search</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Photos' filter.
-2. Tap on a photo result.</t>
+          <t>1. Open advanced search.
+2. Select 'Documents' filter.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the image message.</t>
+          <t>Empty state message should display (e.g., 'No documents found').</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>AS_016</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="n"/>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Verify photo preview from search results</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Photos' filter.
-2. Long press or preview a photo.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Full-size photo preview should open.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AS_017</t>
+          <t>AS_013</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1083,12 +987,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>User is logged in with no image messages</t>
+          <t>User is logged in and has image messages in conversations</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Verify empty state for photos search</t>
+          <t>Verify photos filter displays image messages</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1099,62 +1003,50 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Empty state message should display (e.g., 'No photos found').</t>
+          <t>All image messages across conversations should display as a grid/list.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AS_018</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Verify Videos Search</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has video messages in conversations</t>
-        </is>
-      </c>
+          <t>AS_014</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Verify videos filter displays video messages</t>
+          <t>Verify photo thumbnails display correctly</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Videos' filter.</t>
+          <t>1. Select 'Photos' filter.
+2. Observe results.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>All video messages across conversations should display in results.</t>
+          <t>Photo thumbnails should load and display correctly with sender and date info.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AS_019</t>
+          <t>AS_015</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -1162,30 +1054,30 @@
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Verify video result shows thumbnail and duration</t>
+          <t>Verify tapping photo result opens conversation</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Videos' filter.
-2. Observe results.</t>
+          <t>1. Select 'Photos' filter.
+2. Tap on a photo result.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Each video result should show thumbnail, play icon, duration, sender, and date.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the image message.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AS_020</t>
+          <t>AS_016</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
@@ -1193,166 +1085,124 @@
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping video result opens conversation</t>
+          <t>Verify photo preview from search results</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Videos' filter.
-2. Tap on a video result.</t>
+          <t>1. Select 'Photos' filter.
+2. Long press or preview a photo.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the video message.</t>
+          <t>Full-size photo preview should open.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>AS_021</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Verify Videos Search</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no video messages</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty state for videos search</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Videos' filter.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Empty state message should display (e.g., 'No videos found').</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>AS_022</t>
+          <t>AS_017</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Verify Links Search</t>
+          <t>Verify Photos Search</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>User is logged in and has messages with links</t>
+          <t>User is logged in with no image messages</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Verify links filter displays messages with URLs</t>
+          <t>Verify empty state for photos search</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
-2. Select 'Links' filter.</t>
+2. Select 'Photos' filter.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>All messages containing URLs across conversations should display.</t>
+          <t>Empty state message should display (e.g., 'No photos found').</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>AS_023</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="n"/>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Verify link result shows URL and preview</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Links' filter.
-2. Observe results.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Each result should show the URL, link preview (title/thumbnail if available), sender, and date.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>AS_024</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
+          <t>AS_018</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Verify Videos Search</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has video messages in conversations</t>
+        </is>
+      </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping link result opens conversation</t>
+          <t>Verify videos filter displays video messages</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Links' filter.
-2. Tap on a link result.</t>
+          <t>1. Open advanced search.
+2. Select 'Videos' filter.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the message with the link.</t>
+          <t>All video messages across conversations should display in results.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1364,38 +1214,26 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AS_025</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Verify Links Search</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no link messages</t>
-        </is>
-      </c>
+          <t>AS_019</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Verify empty state for links search</t>
+          <t>Verify video result shows thumbnail and duration</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Links' filter.</t>
+          <t>1. Select 'Videos' filter.
+2. Observe results.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Empty state message should display (e.g., 'No links found').</t>
+          <t>Each video result should show thumbnail, play icon, duration, sender, and date.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1407,39 +1245,26 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>AS_026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Verify Text Message Search</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has text messages</t>
-        </is>
-      </c>
+          <t>AS_020</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Verify text search returns matching messages</t>
+          <t>Verify tapping video result opens conversation</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Text Message' filter.
-3. Type a keyword.</t>
+          <t>1. Select 'Videos' filter.
+2. Tap on a video result.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Messages containing the keyword should display in results.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the video message.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1449,120 +1274,103 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>AS_027</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="n"/>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Verify text search is case-insensitive</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for 'Hello'.
-2. Search for 'hello'.</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Both searches should return the same results.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>AS_028</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
+          <t>AS_021</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Verify Videos Search</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no video messages</t>
+        </is>
+      </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Verify text search highlights matching text</t>
+          <t>Verify empty state for videos search</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1. Search for a keyword.
-2. Observe results.</t>
+          <t>1. Open advanced search.
+2. Select 'Videos' filter.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Matching keyword should be highlighted in the search results.</t>
+          <t>Empty state message should display (e.g., 'No videos found').</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Medium / Low</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>AS_029</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="n"/>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Verify partial text search</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for partial word (e.g., 'hel' for 'hello').</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Messages containing words starting with or containing the partial text should display.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>AS_030</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
+          <t>AS_022</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Verify Links Search</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has messages with links</t>
+        </is>
+      </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping text result opens conversation</t>
+          <t>Verify links filter displays messages with URLs</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>1. Search for a keyword.
-2. Tap on a result.</t>
+          <t>1. Open advanced search.
+2. Select 'Links' filter.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the matching message.</t>
+          <t>All messages containing URLs across conversations should display.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -1574,38 +1382,26 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AS_031</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Verify Text Message Search</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in</t>
-        </is>
-      </c>
+          <t>AS_023</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Verify no results for non-matching search</t>
+          <t>Verify link result shows URL and preview</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Search for a random string that doesn't exist.</t>
+          <t>1. Select 'Links' filter.
+2. Observe results.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Empty state should display (e.g., 'No results found').</t>
+          <t>Each result should show the URL, link preview (title/thumbnail if available), sender, and date.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -1617,7 +1413,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AS_032</t>
+          <t>AS_024</t>
         </is>
       </c>
       <c r="B33" s="2" t="n"/>
@@ -1625,52 +1421,376 @@
       <c r="D33" s="2" t="n"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
+          <t>Verify tapping link result opens conversation</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>1. Select 'Links' filter.
+2. Tap on a link result.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Should navigate to the conversation and highlight/scroll to the message with the link.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>AS_025</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Verify Links Search</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no link messages</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for links search</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Links' filter.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No links found').</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>AS_026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Verify Text Message Search</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has text messages</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Verify text search returns matching messages</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Text Message' filter.
+3. Type a keyword.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Messages containing the keyword should display in results.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>AS_027</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Verify text search is case-insensitive</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for 'Hello'.
+2. Search for 'hello'.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Both searches should return the same results.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>AS_028</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Verify text search highlights matching text</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a keyword.
+2. Observe results.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Matching keyword should be highlighted in the search results.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>AS_029</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Verify partial text search</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for partial word (e.g., 'hel' for 'hello').</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Messages containing words starting with or containing the partial text should display.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>AS_030</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Verify tapping text result opens conversation</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a keyword.
+2. Tap on a result.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Should navigate to the conversation and highlight/scroll to the matching message.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AS_031</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Verify Text Message Search</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Verify no results for non-matching search</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Search for a random string that doesn't exist.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Empty state should display (e.g., 'No results found').</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>AS_032</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>Verify search with special characters</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>1. Search for special characters (e.g., '@#$%').</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Search should handle special characters gracefully without errors.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Low / Medium</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>AS_033</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Verify Advanced Search General</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>User is logged in</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Verify switching between search filters</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
 2. Select 'Photos'.
@@ -1678,87 +1798,97 @@
 4. Switch to 'Documents'.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Results should update correctly when switching between filters.</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>AS_034</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Verify search results pagination/infinite scroll</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search with many results.
 2. Scroll down.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>More results should load as user scrolls. Loading indicator should appear.</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>AS_035</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Verify Advanced Search General</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>User is logged in, network disconnected</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>Verify advanced search fails gracefully without network</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>1. Disconnect network.
 2. Open advanced search.
 3. Try to search.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Appropriate error message should display indicating network issue.</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
@@ -2266,7 +2396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2454,64 +2584,74 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>AS_048</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Verify search during high server load</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>1. Perform search during peak usage.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Search should complete (may be slower) or show timeout message. No crash.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Medium / High</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AS_049</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n"/>
+          <t>AS_048</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>Verify search during high server load</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1. Perform search during peak usage.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Search should complete (may be slower) or show timeout message. No crash.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>AS_049</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>Verify rapid consecutive searches</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>1. Type and search rapidly, changing keywords every second.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>App should debounce requests. Only latest search results should display. No race conditions.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Medium / High</t>
         </is>

</xml_diff>

<commit_message>
Reorder: all Positive test cases first, blank row separator, then all Negative test cases in every sheet
</commit_message>
<xml_diff>
--- a/Advanced_Search/Advanced_Search_Test_Cases.xlsx
+++ b/Advanced_Search/Advanced_Search_Test_Cases.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -739,50 +739,71 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AS_009</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Verify Documents Search</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has document messages in conversations</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Verify documents filter displays document messages</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Documents' filter.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>All document/file messages across conversations should display in results.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AS_008</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Verify Audio Search</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no audio messages</t>
-        </is>
-      </c>
+          <t>AS_010</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Verify empty state for audio search</t>
+          <t>Verify document result shows file details</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Audio' filter.</t>
+          <t>1. Select 'Documents' filter.
+2. Observe results.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Empty state message should display (e.g., 'No audio messages found').</t>
+          <t>Each result should show file name, file type icon, size, sender, and date.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -792,19 +813,40 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AS_011</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Verify tapping document result opens conversation</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1. Select 'Documents' filter.
+2. Tap on a document result.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Should navigate to the conversation and highlight/scroll to the document message.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AS_009</t>
+          <t>AS_013</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -814,28 +856,28 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Verify Documents Search</t>
+          <t>Verify Photos Search</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>User is logged in and has document messages in conversations</t>
+          <t>User is logged in and has image messages in conversations</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Verify documents filter displays document messages</t>
+          <t>Verify photos filter displays image messages</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
-2. Select 'Documents' filter.</t>
+2. Select 'Photos' filter.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>All document/file messages across conversations should display in results.</t>
+          <t>All image messages across conversations should display as a grid/list.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -847,7 +889,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AS_010</t>
+          <t>AS_014</t>
         </is>
       </c>
       <c r="B13" s="2" t="n"/>
@@ -855,18 +897,18 @@
       <c r="D13" s="2" t="n"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Verify document result shows file details</t>
+          <t>Verify photo thumbnails display correctly</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Documents' filter.
+          <t>1. Select 'Photos' filter.
 2. Observe results.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Each result should show file name, file type icon, size, sender, and date.</t>
+          <t>Photo thumbnails should load and display correctly with sender and date info.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -878,7 +920,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>AS_011</t>
+          <t>AS_015</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -886,18 +928,18 @@
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping document result opens conversation</t>
+          <t>Verify tapping photo result opens conversation</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Documents' filter.
-2. Tap on a document result.</t>
+          <t>1. Select 'Photos' filter.
+2. Tap on a photo result.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the document message.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the image message.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -907,103 +949,133 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>AS_016</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="n"/>
       <c r="C15" s="2" t="n"/>
       <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Verify photo preview from search results</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1. Select 'Photos' filter.
+2. Long press or preview a photo.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Full-size photo preview should open.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>AS_012</t>
+          <t>AS_018</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Verify Documents Search</t>
+          <t>Verify Videos Search</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>User is logged in with no document messages</t>
+          <t>User is logged in and has video messages in conversations</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Verify empty state for documents search</t>
+          <t>Verify videos filter displays video messages</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
-2. Select 'Documents' filter.</t>
+2. Select 'Videos' filter.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Empty state message should display (e.g., 'No documents found').</t>
+          <t>All video messages across conversations should display in results.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AS_019</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="n"/>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Verify video result shows thumbnail and duration</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>1. Select 'Videos' filter.
+2. Observe results.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Each video result should show thumbnail, play icon, duration, sender, and date.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>AS_013</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Verify Photos Search</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has image messages in conversations</t>
-        </is>
-      </c>
+          <t>AS_020</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Verify photos filter displays image messages</t>
+          <t>Verify tapping video result opens conversation</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Photos' filter.</t>
+          <t>1. Select 'Videos' filter.
+2. Tap on a video result.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>All image messages across conversations should display as a grid/list.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the video message.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1015,38 +1087,50 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>AS_014</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
+          <t>AS_022</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Verify Links Search</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has messages with links</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Verify photo thumbnails display correctly</t>
+          <t>Verify links filter displays messages with URLs</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Photos' filter.
-2. Observe results.</t>
+          <t>1. Open advanced search.
+2. Select 'Links' filter.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Photo thumbnails should load and display correctly with sender and date info.</t>
+          <t>All messages containing URLs across conversations should display.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>AS_015</t>
+          <t>AS_023</t>
         </is>
       </c>
       <c r="B20" s="2" t="n"/>
@@ -1054,30 +1138,30 @@
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping photo result opens conversation</t>
+          <t>Verify link result shows URL and preview</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Photos' filter.
-2. Tap on a photo result.</t>
+          <t>1. Select 'Links' filter.
+2. Observe results.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Should navigate to the conversation and highlight/scroll to the image message.</t>
+          <t>Each result should show the URL, link preview (title/thumbnail if available), sender, and date.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AS_016</t>
+          <t>AS_024</t>
         </is>
       </c>
       <c r="B21" s="2" t="n"/>
@@ -1085,71 +1169,93 @@
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Verify photo preview from search results</t>
+          <t>Verify tapping link result opens conversation</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Photos' filter.
-2. Long press or preview a photo.</t>
+          <t>1. Select 'Links' filter.
+2. Tap on a link result.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Full-size photo preview should open.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the message with the link.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>AS_026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Verify Text Message Search</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and has text messages</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Verify text search returns matching messages</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Text Message' filter.
+3. Type a keyword.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Messages containing the keyword should display in results.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>AS_017</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Verify Photos Search</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no image messages</t>
-        </is>
-      </c>
+          <t>AS_027</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Verify empty state for photos search</t>
+          <t>Verify text search is case-insensitive</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Photos' filter.</t>
+          <t>1. Search for 'Hello'.
+2. Search for 'hello'.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Empty state message should display (e.g., 'No photos found').</t>
+          <t>Both searches should return the same results.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1159,62 +1265,70 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>AS_028</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Verify text search highlights matching text</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for a keyword.
+2. Observe results.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Matching keyword should be highlighted in the search results.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Low</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>AS_018</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Verify Videos Search</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has video messages in conversations</t>
-        </is>
-      </c>
+          <t>AS_029</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Verify videos filter displays video messages</t>
+          <t>Verify partial text search</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>1. Open advanced search.
-2. Select 'Videos' filter.</t>
+          <t>1. Search for partial word (e.g., 'hel' for 'hello').</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>All video messages across conversations should display in results.</t>
+          <t>Messages containing words starting with or containing the partial text should display.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AS_019</t>
+          <t>AS_030</t>
         </is>
       </c>
       <c r="B26" s="2" t="n"/>
@@ -1222,575 +1336,53 @@
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Verify video result shows thumbnail and duration</t>
+          <t>Verify tapping text result opens conversation</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>1. Select 'Videos' filter.
-2. Observe results.</t>
+          <t>1. Search for a keyword.
+2. Tap on a result.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Each video result should show thumbnail, play icon, duration, sender, and date.</t>
+          <t>Should navigate to the conversation and highlight/scroll to the matching message.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>AS_020</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
+          <t>AS_033</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Verify Advanced Search General</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Verify tapping video result opens conversation</t>
+          <t>Verify switching between search filters</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Videos' filter.
-2. Tap on a video result.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Should navigate to the conversation and highlight/scroll to the video message.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>AS_021</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Verify Videos Search</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no video messages</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty state for videos search</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Videos' filter.</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Empty state message should display (e.g., 'No videos found').</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>AS_022</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Verify Links Search</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has messages with links</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Verify links filter displays messages with URLs</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Links' filter.</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>All messages containing URLs across conversations should display.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>AS_023</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Verify link result shows URL and preview</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Links' filter.
-2. Observe results.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Each result should show the URL, link preview (title/thumbnail if available), sender, and date.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>AS_024</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Verify tapping link result opens conversation</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>1. Select 'Links' filter.
-2. Tap on a link result.</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Should navigate to the conversation and highlight/scroll to the message with the link.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>AS_025</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Verify Links Search</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in with no link messages</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Verify empty state for links search</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Links' filter.</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Empty state message should display (e.g., 'No links found').</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>AS_026</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Verify Text Message Search</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and has text messages</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Verify text search returns matching messages</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Select 'Text Message' filter.
-3. Type a keyword.</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Messages containing the keyword should display in results.</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>AS_027</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Verify text search is case-insensitive</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for 'Hello'.
-2. Search for 'hello'.</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Both searches should return the same results.</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>AS_028</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Verify text search highlights matching text</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for a keyword.
-2. Observe results.</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Matching keyword should be highlighted in the search results.</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>AS_029</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Verify partial text search</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for partial word (e.g., 'hel' for 'hello').</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Messages containing words starting with or containing the partial text should display.</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>AS_030</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Verify tapping text result opens conversation</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for a keyword.
-2. Tap on a result.</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Should navigate to the conversation and highlight/scroll to the matching message.</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>AS_031</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Verify Text Message Search</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Verify no results for non-matching search</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>1. Open advanced search.
-2. Search for a random string that doesn't exist.</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Empty state should display (e.g., 'No results found').</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>AS_032</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Verify search with special characters</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>1. Search for special characters (e.g., '@#$%').</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Search should handle special characters gracefully without errors.</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Low / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>AS_033</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Verify Advanced Search General</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Verify switching between search filters</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search.
 2. Select 'Photos'.
@@ -1798,97 +1390,385 @@
 4. Switch to 'Documents'.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Results should update correctly when switching between filters.</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>AS_034</t>
         </is>
       </c>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Verify search results pagination/infinite scroll</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1. Open advanced search with many results.
 2. Scroll down.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>More results should load as user scrolls. Loading indicator should appear.</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>AS_008</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Verify Audio Search</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no audio messages</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for audio search</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Audio' filter.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No audio messages found').</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>AS_012</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Verify Documents Search</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no document messages</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for documents search</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Documents' filter.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No documents found').</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>AS_017</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Verify Photos Search</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no image messages</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for photos search</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Photos' filter.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No photos found').</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>AS_021</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Verify Videos Search</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no video messages</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for videos search</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Videos' filter.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No videos found').</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>AS_025</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Verify Links Search</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in with no link messages</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Verify empty state for links search</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Select 'Links' filter.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Empty state message should display (e.g., 'No links found').</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>AS_031</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Verify Text Message Search</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Verify no results for non-matching search</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>1. Open advanced search.
+2. Search for a random string that doesn't exist.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Empty state should display (e.g., 'No results found').</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>AS_032</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Verify search with special characters</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>1. Search for special characters (e.g., '@#$%').</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Search should handle special characters gracefully without errors.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Low / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>AS_035</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Verify Advanced Search General</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>User is logged in, network disconnected</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Verify advanced search fails gracefully without network</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>1. Disconnect network.
 2. Open advanced search.
 3. Try to search.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Appropriate error message should display indicating network issue.</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>High / High</t>
         </is>

</xml_diff>